<commit_message>
Can be edit inside the webpage
</commit_message>
<xml_diff>
--- a/itinerary.xlsx
+++ b/itinerary.xlsx
@@ -435,17 +435,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H300"/>
+  <dimension ref="A1:I300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,30 +462,35 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>类别</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>地点</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>城市</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>地址</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>纬度</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>经度</t>
         </is>
@@ -501,28 +507,33 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>北京首都国际机场 T3</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>北京市顺义区首都机场路</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>示例：抵达后坐机场快轨进城</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>40.0799</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>116.6031</v>
       </c>
     </row>
@@ -537,102 +548,97 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>晚餐</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>王府井步行街</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>北京市东城区王府井大街</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>示例：晚饭和夜市小吃</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>示例：夜市小吃</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>39.9139</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>116.4175</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>天安门广场</t>
+          <t>住宿</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>北京王府井附近酒店</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>北京市东城区东长安街</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>示例：带护照，过安检</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>39.9055</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>116.3976</v>
-      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>示例：住宿</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
+      <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>故宫博物院</t>
+          <t>标题</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>天安门-故宫-景山一日游</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>北京市东城区景山前街4号</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>示例：需提前实名预约，带护照</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>39.9163</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>116.3972</v>
-      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>示例：整天步行，穿舒服的鞋，带水</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -640,1596 +646,1717 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>景山公园</t>
+          <t>早餐</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>酒店含早</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>北京市西城区景山西街44号</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>示例：爬到万春亭看故宫全景</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>39.9254</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>116.3957</v>
-      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>八达岭长城</t>
+          <t>景点</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>天安门广场</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>北京市延庆区八达岭镇</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>示例：从黄土店站坐 S2 线，路上约 1 小时</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>40.3598</v>
+          <t>北京市东城区东长安街</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>示例：带护照，过安检</t>
+        </is>
       </c>
       <c r="H7" s="3" t="n">
-        <v>116.02</v>
+        <v>39.9055</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>116.3976</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>北京西站</t>
+          <t>景点</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>故宫博物院</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>北京市丰台区莲花池东路118号</t>
-        </is>
-      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>示例：坐高铁去西安，提前 1 小时到站</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>39.8946</v>
+          <t>北京市东城区景山前街4号</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>示例：需提前实名预约，带护照</t>
+        </is>
       </c>
       <c r="H8" s="3" t="n">
-        <v>116.322</v>
+        <v>39.9163</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>116.3972</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>景山公园</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>北京市西城区景山西街44号</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>示例：爬到万春亭看故宫全景</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>39.9254</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>116.3957</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>景点</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>八达岭长城</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>北京市延庆区八达岭镇</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>示例：从黄土店站坐 S2 线，路上约 1 小时</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>40.3598</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>116.02</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>交通</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>北京西站</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>北京市丰台区莲花池东路118号</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>示例：坐高铁去西安，提前 1 小时到站</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>39.8946</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>116.322</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>晚餐</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>回民街</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>西安</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>西安市莲湖区北院门</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>示例：没填经纬度，地图按城市估算位置</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="2" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="2" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="2" t="n"/>
-      <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="2" t="n"/>
-      <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="2" t="n"/>
-      <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="2" t="n"/>
-      <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="2" t="n"/>
-      <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="2" t="n"/>
-      <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="2" t="n"/>
-      <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="2" t="n"/>
-      <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="2" t="n"/>
-      <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="2" t="n"/>
-      <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="2" t="n"/>
-      <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="2" t="n"/>
-      <c r="G23" s="3" t="n"/>
       <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="2" t="n"/>
-      <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="2" t="n"/>
-      <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="2" t="n"/>
-      <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="B27" s="2" t="n"/>
-      <c r="G27" s="3" t="n"/>
       <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="2" t="n"/>
-      <c r="G28" s="3" t="n"/>
       <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="2" t="n"/>
-      <c r="G29" s="3" t="n"/>
       <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="2" t="n"/>
-      <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="n"/>
+      <c r="I30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="2" t="n"/>
-      <c r="G31" s="3" t="n"/>
       <c r="H31" s="3" t="n"/>
+      <c r="I31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="2" t="n"/>
-      <c r="G32" s="3" t="n"/>
       <c r="H32" s="3" t="n"/>
+      <c r="I32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="2" t="n"/>
-      <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="2" t="n"/>
-      <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="2" t="n"/>
-      <c r="G35" s="3" t="n"/>
       <c r="H35" s="3" t="n"/>
+      <c r="I35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="2" t="n"/>
-      <c r="G36" s="3" t="n"/>
       <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="2" t="n"/>
-      <c r="G37" s="3" t="n"/>
       <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="2" t="n"/>
-      <c r="G38" s="3" t="n"/>
       <c r="H38" s="3" t="n"/>
+      <c r="I38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="2" t="n"/>
-      <c r="G39" s="3" t="n"/>
       <c r="H39" s="3" t="n"/>
+      <c r="I39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="2" t="n"/>
-      <c r="G40" s="3" t="n"/>
       <c r="H40" s="3" t="n"/>
+      <c r="I40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="2" t="n"/>
-      <c r="G41" s="3" t="n"/>
       <c r="H41" s="3" t="n"/>
+      <c r="I41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="2" t="n"/>
-      <c r="G42" s="3" t="n"/>
       <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="2" t="n"/>
-      <c r="G43" s="3" t="n"/>
       <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="2" t="n"/>
-      <c r="G44" s="3" t="n"/>
       <c r="H44" s="3" t="n"/>
+      <c r="I44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="2" t="n"/>
-      <c r="G45" s="3" t="n"/>
       <c r="H45" s="3" t="n"/>
+      <c r="I45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="B46" s="2" t="n"/>
-      <c r="G46" s="3" t="n"/>
       <c r="H46" s="3" t="n"/>
+      <c r="I46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="2" t="n"/>
-      <c r="G47" s="3" t="n"/>
       <c r="H47" s="3" t="n"/>
+      <c r="I47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="B48" s="2" t="n"/>
-      <c r="G48" s="3" t="n"/>
       <c r="H48" s="3" t="n"/>
+      <c r="I48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="B49" s="2" t="n"/>
-      <c r="G49" s="3" t="n"/>
       <c r="H49" s="3" t="n"/>
+      <c r="I49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="B50" s="2" t="n"/>
-      <c r="G50" s="3" t="n"/>
       <c r="H50" s="3" t="n"/>
+      <c r="I50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="B51" s="2" t="n"/>
-      <c r="G51" s="3" t="n"/>
       <c r="H51" s="3" t="n"/>
+      <c r="I51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="2" t="n"/>
-      <c r="G52" s="3" t="n"/>
       <c r="H52" s="3" t="n"/>
+      <c r="I52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="B53" s="2" t="n"/>
-      <c r="G53" s="3" t="n"/>
       <c r="H53" s="3" t="n"/>
+      <c r="I53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="B54" s="2" t="n"/>
-      <c r="G54" s="3" t="n"/>
       <c r="H54" s="3" t="n"/>
+      <c r="I54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="B55" s="2" t="n"/>
-      <c r="G55" s="3" t="n"/>
       <c r="H55" s="3" t="n"/>
+      <c r="I55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="B56" s="2" t="n"/>
-      <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="n"/>
+      <c r="I56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="B57" s="2" t="n"/>
-      <c r="G57" s="3" t="n"/>
       <c r="H57" s="3" t="n"/>
+      <c r="I57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="B58" s="2" t="n"/>
-      <c r="G58" s="3" t="n"/>
       <c r="H58" s="3" t="n"/>
+      <c r="I58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="B59" s="2" t="n"/>
-      <c r="G59" s="3" t="n"/>
       <c r="H59" s="3" t="n"/>
+      <c r="I59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="2" t="n"/>
-      <c r="G60" s="3" t="n"/>
       <c r="H60" s="3" t="n"/>
+      <c r="I60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="B61" s="2" t="n"/>
-      <c r="G61" s="3" t="n"/>
       <c r="H61" s="3" t="n"/>
+      <c r="I61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="2" t="n"/>
-      <c r="G62" s="3" t="n"/>
       <c r="H62" s="3" t="n"/>
+      <c r="I62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="B63" s="2" t="n"/>
-      <c r="G63" s="3" t="n"/>
       <c r="H63" s="3" t="n"/>
+      <c r="I63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="B64" s="2" t="n"/>
-      <c r="G64" s="3" t="n"/>
       <c r="H64" s="3" t="n"/>
+      <c r="I64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="2" t="n"/>
-      <c r="G65" s="3" t="n"/>
       <c r="H65" s="3" t="n"/>
+      <c r="I65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="2" t="n"/>
-      <c r="G66" s="3" t="n"/>
       <c r="H66" s="3" t="n"/>
+      <c r="I66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="B67" s="2" t="n"/>
-      <c r="G67" s="3" t="n"/>
       <c r="H67" s="3" t="n"/>
+      <c r="I67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="B68" s="2" t="n"/>
-      <c r="G68" s="3" t="n"/>
       <c r="H68" s="3" t="n"/>
+      <c r="I68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="B69" s="2" t="n"/>
-      <c r="G69" s="3" t="n"/>
       <c r="H69" s="3" t="n"/>
+      <c r="I69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="2" t="n"/>
-      <c r="G70" s="3" t="n"/>
       <c r="H70" s="3" t="n"/>
+      <c r="I70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="2" t="n"/>
-      <c r="G71" s="3" t="n"/>
       <c r="H71" s="3" t="n"/>
+      <c r="I71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="2" t="n"/>
-      <c r="G72" s="3" t="n"/>
       <c r="H72" s="3" t="n"/>
+      <c r="I72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="B73" s="2" t="n"/>
-      <c r="G73" s="3" t="n"/>
       <c r="H73" s="3" t="n"/>
+      <c r="I73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="B74" s="2" t="n"/>
-      <c r="G74" s="3" t="n"/>
       <c r="H74" s="3" t="n"/>
+      <c r="I74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="2" t="n"/>
-      <c r="G75" s="3" t="n"/>
       <c r="H75" s="3" t="n"/>
+      <c r="I75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="B76" s="2" t="n"/>
-      <c r="G76" s="3" t="n"/>
       <c r="H76" s="3" t="n"/>
+      <c r="I76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="B77" s="2" t="n"/>
-      <c r="G77" s="3" t="n"/>
       <c r="H77" s="3" t="n"/>
+      <c r="I77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="B78" s="2" t="n"/>
-      <c r="G78" s="3" t="n"/>
       <c r="H78" s="3" t="n"/>
+      <c r="I78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="B79" s="2" t="n"/>
-      <c r="G79" s="3" t="n"/>
       <c r="H79" s="3" t="n"/>
+      <c r="I79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="B80" s="2" t="n"/>
-      <c r="G80" s="3" t="n"/>
       <c r="H80" s="3" t="n"/>
+      <c r="I80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="B81" s="2" t="n"/>
-      <c r="G81" s="3" t="n"/>
       <c r="H81" s="3" t="n"/>
+      <c r="I81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="2" t="n"/>
-      <c r="G82" s="3" t="n"/>
       <c r="H82" s="3" t="n"/>
+      <c r="I82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="2" t="n"/>
-      <c r="G83" s="3" t="n"/>
       <c r="H83" s="3" t="n"/>
+      <c r="I83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="B84" s="2" t="n"/>
-      <c r="G84" s="3" t="n"/>
       <c r="H84" s="3" t="n"/>
+      <c r="I84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="B85" s="2" t="n"/>
-      <c r="G85" s="3" t="n"/>
       <c r="H85" s="3" t="n"/>
+      <c r="I85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="B86" s="2" t="n"/>
-      <c r="G86" s="3" t="n"/>
       <c r="H86" s="3" t="n"/>
+      <c r="I86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="B87" s="2" t="n"/>
-      <c r="G87" s="3" t="n"/>
       <c r="H87" s="3" t="n"/>
+      <c r="I87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="B88" s="2" t="n"/>
-      <c r="G88" s="3" t="n"/>
       <c r="H88" s="3" t="n"/>
+      <c r="I88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="B89" s="2" t="n"/>
-      <c r="G89" s="3" t="n"/>
       <c r="H89" s="3" t="n"/>
+      <c r="I89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="B90" s="2" t="n"/>
-      <c r="G90" s="3" t="n"/>
       <c r="H90" s="3" t="n"/>
+      <c r="I90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="B91" s="2" t="n"/>
-      <c r="G91" s="3" t="n"/>
       <c r="H91" s="3" t="n"/>
+      <c r="I91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="B92" s="2" t="n"/>
-      <c r="G92" s="3" t="n"/>
       <c r="H92" s="3" t="n"/>
+      <c r="I92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="B93" s="2" t="n"/>
-      <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="n"/>
+      <c r="I93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="B94" s="2" t="n"/>
-      <c r="G94" s="3" t="n"/>
       <c r="H94" s="3" t="n"/>
+      <c r="I94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="B95" s="2" t="n"/>
-      <c r="G95" s="3" t="n"/>
       <c r="H95" s="3" t="n"/>
+      <c r="I95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="B96" s="2" t="n"/>
-      <c r="G96" s="3" t="n"/>
       <c r="H96" s="3" t="n"/>
+      <c r="I96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="B97" s="2" t="n"/>
-      <c r="G97" s="3" t="n"/>
       <c r="H97" s="3" t="n"/>
+      <c r="I97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="2" t="n"/>
-      <c r="G98" s="3" t="n"/>
       <c r="H98" s="3" t="n"/>
+      <c r="I98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="B99" s="2" t="n"/>
-      <c r="G99" s="3" t="n"/>
       <c r="H99" s="3" t="n"/>
+      <c r="I99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="B100" s="2" t="n"/>
-      <c r="G100" s="3" t="n"/>
       <c r="H100" s="3" t="n"/>
+      <c r="I100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="B101" s="2" t="n"/>
-      <c r="G101" s="3" t="n"/>
       <c r="H101" s="3" t="n"/>
+      <c r="I101" s="3" t="n"/>
     </row>
     <row r="102">
       <c r="B102" s="2" t="n"/>
-      <c r="G102" s="3" t="n"/>
       <c r="H102" s="3" t="n"/>
+      <c r="I102" s="3" t="n"/>
     </row>
     <row r="103">
       <c r="B103" s="2" t="n"/>
-      <c r="G103" s="3" t="n"/>
       <c r="H103" s="3" t="n"/>
+      <c r="I103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="B104" s="2" t="n"/>
-      <c r="G104" s="3" t="n"/>
       <c r="H104" s="3" t="n"/>
+      <c r="I104" s="3" t="n"/>
     </row>
     <row r="105">
       <c r="B105" s="2" t="n"/>
-      <c r="G105" s="3" t="n"/>
       <c r="H105" s="3" t="n"/>
+      <c r="I105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="B106" s="2" t="n"/>
-      <c r="G106" s="3" t="n"/>
       <c r="H106" s="3" t="n"/>
+      <c r="I106" s="3" t="n"/>
     </row>
     <row r="107">
       <c r="B107" s="2" t="n"/>
-      <c r="G107" s="3" t="n"/>
       <c r="H107" s="3" t="n"/>
+      <c r="I107" s="3" t="n"/>
     </row>
     <row r="108">
       <c r="B108" s="2" t="n"/>
-      <c r="G108" s="3" t="n"/>
       <c r="H108" s="3" t="n"/>
+      <c r="I108" s="3" t="n"/>
     </row>
     <row r="109">
       <c r="B109" s="2" t="n"/>
-      <c r="G109" s="3" t="n"/>
       <c r="H109" s="3" t="n"/>
+      <c r="I109" s="3" t="n"/>
     </row>
     <row r="110">
       <c r="B110" s="2" t="n"/>
-      <c r="G110" s="3" t="n"/>
       <c r="H110" s="3" t="n"/>
+      <c r="I110" s="3" t="n"/>
     </row>
     <row r="111">
       <c r="B111" s="2" t="n"/>
-      <c r="G111" s="3" t="n"/>
       <c r="H111" s="3" t="n"/>
+      <c r="I111" s="3" t="n"/>
     </row>
     <row r="112">
       <c r="B112" s="2" t="n"/>
-      <c r="G112" s="3" t="n"/>
       <c r="H112" s="3" t="n"/>
+      <c r="I112" s="3" t="n"/>
     </row>
     <row r="113">
       <c r="B113" s="2" t="n"/>
-      <c r="G113" s="3" t="n"/>
       <c r="H113" s="3" t="n"/>
+      <c r="I113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="B114" s="2" t="n"/>
-      <c r="G114" s="3" t="n"/>
       <c r="H114" s="3" t="n"/>
+      <c r="I114" s="3" t="n"/>
     </row>
     <row r="115">
       <c r="B115" s="2" t="n"/>
-      <c r="G115" s="3" t="n"/>
       <c r="H115" s="3" t="n"/>
+      <c r="I115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="B116" s="2" t="n"/>
-      <c r="G116" s="3" t="n"/>
       <c r="H116" s="3" t="n"/>
+      <c r="I116" s="3" t="n"/>
     </row>
     <row r="117">
       <c r="B117" s="2" t="n"/>
-      <c r="G117" s="3" t="n"/>
       <c r="H117" s="3" t="n"/>
+      <c r="I117" s="3" t="n"/>
     </row>
     <row r="118">
       <c r="B118" s="2" t="n"/>
-      <c r="G118" s="3" t="n"/>
       <c r="H118" s="3" t="n"/>
+      <c r="I118" s="3" t="n"/>
     </row>
     <row r="119">
       <c r="B119" s="2" t="n"/>
-      <c r="G119" s="3" t="n"/>
       <c r="H119" s="3" t="n"/>
+      <c r="I119" s="3" t="n"/>
     </row>
     <row r="120">
       <c r="B120" s="2" t="n"/>
-      <c r="G120" s="3" t="n"/>
       <c r="H120" s="3" t="n"/>
+      <c r="I120" s="3" t="n"/>
     </row>
     <row r="121">
       <c r="B121" s="2" t="n"/>
-      <c r="G121" s="3" t="n"/>
       <c r="H121" s="3" t="n"/>
+      <c r="I121" s="3" t="n"/>
     </row>
     <row r="122">
       <c r="B122" s="2" t="n"/>
-      <c r="G122" s="3" t="n"/>
       <c r="H122" s="3" t="n"/>
+      <c r="I122" s="3" t="n"/>
     </row>
     <row r="123">
       <c r="B123" s="2" t="n"/>
-      <c r="G123" s="3" t="n"/>
       <c r="H123" s="3" t="n"/>
+      <c r="I123" s="3" t="n"/>
     </row>
     <row r="124">
       <c r="B124" s="2" t="n"/>
-      <c r="G124" s="3" t="n"/>
       <c r="H124" s="3" t="n"/>
+      <c r="I124" s="3" t="n"/>
     </row>
     <row r="125">
       <c r="B125" s="2" t="n"/>
-      <c r="G125" s="3" t="n"/>
       <c r="H125" s="3" t="n"/>
+      <c r="I125" s="3" t="n"/>
     </row>
     <row r="126">
       <c r="B126" s="2" t="n"/>
-      <c r="G126" s="3" t="n"/>
       <c r="H126" s="3" t="n"/>
+      <c r="I126" s="3" t="n"/>
     </row>
     <row r="127">
       <c r="B127" s="2" t="n"/>
-      <c r="G127" s="3" t="n"/>
       <c r="H127" s="3" t="n"/>
+      <c r="I127" s="3" t="n"/>
     </row>
     <row r="128">
       <c r="B128" s="2" t="n"/>
-      <c r="G128" s="3" t="n"/>
       <c r="H128" s="3" t="n"/>
+      <c r="I128" s="3" t="n"/>
     </row>
     <row r="129">
       <c r="B129" s="2" t="n"/>
-      <c r="G129" s="3" t="n"/>
       <c r="H129" s="3" t="n"/>
+      <c r="I129" s="3" t="n"/>
     </row>
     <row r="130">
       <c r="B130" s="2" t="n"/>
-      <c r="G130" s="3" t="n"/>
       <c r="H130" s="3" t="n"/>
+      <c r="I130" s="3" t="n"/>
     </row>
     <row r="131">
       <c r="B131" s="2" t="n"/>
-      <c r="G131" s="3" t="n"/>
       <c r="H131" s="3" t="n"/>
+      <c r="I131" s="3" t="n"/>
     </row>
     <row r="132">
       <c r="B132" s="2" t="n"/>
-      <c r="G132" s="3" t="n"/>
       <c r="H132" s="3" t="n"/>
+      <c r="I132" s="3" t="n"/>
     </row>
     <row r="133">
       <c r="B133" s="2" t="n"/>
-      <c r="G133" s="3" t="n"/>
       <c r="H133" s="3" t="n"/>
+      <c r="I133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="B134" s="2" t="n"/>
-      <c r="G134" s="3" t="n"/>
       <c r="H134" s="3" t="n"/>
+      <c r="I134" s="3" t="n"/>
     </row>
     <row r="135">
       <c r="B135" s="2" t="n"/>
-      <c r="G135" s="3" t="n"/>
       <c r="H135" s="3" t="n"/>
+      <c r="I135" s="3" t="n"/>
     </row>
     <row r="136">
       <c r="B136" s="2" t="n"/>
-      <c r="G136" s="3" t="n"/>
       <c r="H136" s="3" t="n"/>
+      <c r="I136" s="3" t="n"/>
     </row>
     <row r="137">
       <c r="B137" s="2" t="n"/>
-      <c r="G137" s="3" t="n"/>
       <c r="H137" s="3" t="n"/>
+      <c r="I137" s="3" t="n"/>
     </row>
     <row r="138">
       <c r="B138" s="2" t="n"/>
-      <c r="G138" s="3" t="n"/>
       <c r="H138" s="3" t="n"/>
+      <c r="I138" s="3" t="n"/>
     </row>
     <row r="139">
       <c r="B139" s="2" t="n"/>
-      <c r="G139" s="3" t="n"/>
       <c r="H139" s="3" t="n"/>
+      <c r="I139" s="3" t="n"/>
     </row>
     <row r="140">
       <c r="B140" s="2" t="n"/>
-      <c r="G140" s="3" t="n"/>
       <c r="H140" s="3" t="n"/>
+      <c r="I140" s="3" t="n"/>
     </row>
     <row r="141">
       <c r="B141" s="2" t="n"/>
-      <c r="G141" s="3" t="n"/>
       <c r="H141" s="3" t="n"/>
+      <c r="I141" s="3" t="n"/>
     </row>
     <row r="142">
       <c r="B142" s="2" t="n"/>
-      <c r="G142" s="3" t="n"/>
       <c r="H142" s="3" t="n"/>
+      <c r="I142" s="3" t="n"/>
     </row>
     <row r="143">
       <c r="B143" s="2" t="n"/>
-      <c r="G143" s="3" t="n"/>
       <c r="H143" s="3" t="n"/>
+      <c r="I143" s="3" t="n"/>
     </row>
     <row r="144">
       <c r="B144" s="2" t="n"/>
-      <c r="G144" s="3" t="n"/>
       <c r="H144" s="3" t="n"/>
+      <c r="I144" s="3" t="n"/>
     </row>
     <row r="145">
       <c r="B145" s="2" t="n"/>
-      <c r="G145" s="3" t="n"/>
       <c r="H145" s="3" t="n"/>
+      <c r="I145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="B146" s="2" t="n"/>
-      <c r="G146" s="3" t="n"/>
       <c r="H146" s="3" t="n"/>
+      <c r="I146" s="3" t="n"/>
     </row>
     <row r="147">
       <c r="B147" s="2" t="n"/>
-      <c r="G147" s="3" t="n"/>
       <c r="H147" s="3" t="n"/>
+      <c r="I147" s="3" t="n"/>
     </row>
     <row r="148">
       <c r="B148" s="2" t="n"/>
-      <c r="G148" s="3" t="n"/>
       <c r="H148" s="3" t="n"/>
+      <c r="I148" s="3" t="n"/>
     </row>
     <row r="149">
       <c r="B149" s="2" t="n"/>
-      <c r="G149" s="3" t="n"/>
       <c r="H149" s="3" t="n"/>
+      <c r="I149" s="3" t="n"/>
     </row>
     <row r="150">
       <c r="B150" s="2" t="n"/>
-      <c r="G150" s="3" t="n"/>
       <c r="H150" s="3" t="n"/>
+      <c r="I150" s="3" t="n"/>
     </row>
     <row r="151">
       <c r="B151" s="2" t="n"/>
-      <c r="G151" s="3" t="n"/>
       <c r="H151" s="3" t="n"/>
+      <c r="I151" s="3" t="n"/>
     </row>
     <row r="152">
       <c r="B152" s="2" t="n"/>
-      <c r="G152" s="3" t="n"/>
       <c r="H152" s="3" t="n"/>
+      <c r="I152" s="3" t="n"/>
     </row>
     <row r="153">
       <c r="B153" s="2" t="n"/>
-      <c r="G153" s="3" t="n"/>
       <c r="H153" s="3" t="n"/>
+      <c r="I153" s="3" t="n"/>
     </row>
     <row r="154">
       <c r="B154" s="2" t="n"/>
-      <c r="G154" s="3" t="n"/>
       <c r="H154" s="3" t="n"/>
+      <c r="I154" s="3" t="n"/>
     </row>
     <row r="155">
       <c r="B155" s="2" t="n"/>
-      <c r="G155" s="3" t="n"/>
       <c r="H155" s="3" t="n"/>
+      <c r="I155" s="3" t="n"/>
     </row>
     <row r="156">
       <c r="B156" s="2" t="n"/>
-      <c r="G156" s="3" t="n"/>
       <c r="H156" s="3" t="n"/>
+      <c r="I156" s="3" t="n"/>
     </row>
     <row r="157">
       <c r="B157" s="2" t="n"/>
-      <c r="G157" s="3" t="n"/>
       <c r="H157" s="3" t="n"/>
+      <c r="I157" s="3" t="n"/>
     </row>
     <row r="158">
       <c r="B158" s="2" t="n"/>
-      <c r="G158" s="3" t="n"/>
       <c r="H158" s="3" t="n"/>
+      <c r="I158" s="3" t="n"/>
     </row>
     <row r="159">
       <c r="B159" s="2" t="n"/>
-      <c r="G159" s="3" t="n"/>
       <c r="H159" s="3" t="n"/>
+      <c r="I159" s="3" t="n"/>
     </row>
     <row r="160">
       <c r="B160" s="2" t="n"/>
-      <c r="G160" s="3" t="n"/>
       <c r="H160" s="3" t="n"/>
+      <c r="I160" s="3" t="n"/>
     </row>
     <row r="161">
       <c r="B161" s="2" t="n"/>
-      <c r="G161" s="3" t="n"/>
       <c r="H161" s="3" t="n"/>
+      <c r="I161" s="3" t="n"/>
     </row>
     <row r="162">
       <c r="B162" s="2" t="n"/>
-      <c r="G162" s="3" t="n"/>
       <c r="H162" s="3" t="n"/>
+      <c r="I162" s="3" t="n"/>
     </row>
     <row r="163">
       <c r="B163" s="2" t="n"/>
-      <c r="G163" s="3" t="n"/>
       <c r="H163" s="3" t="n"/>
+      <c r="I163" s="3" t="n"/>
     </row>
     <row r="164">
       <c r="B164" s="2" t="n"/>
-      <c r="G164" s="3" t="n"/>
       <c r="H164" s="3" t="n"/>
+      <c r="I164" s="3" t="n"/>
     </row>
     <row r="165">
       <c r="B165" s="2" t="n"/>
-      <c r="G165" s="3" t="n"/>
       <c r="H165" s="3" t="n"/>
+      <c r="I165" s="3" t="n"/>
     </row>
     <row r="166">
       <c r="B166" s="2" t="n"/>
-      <c r="G166" s="3" t="n"/>
       <c r="H166" s="3" t="n"/>
+      <c r="I166" s="3" t="n"/>
     </row>
     <row r="167">
       <c r="B167" s="2" t="n"/>
-      <c r="G167" s="3" t="n"/>
       <c r="H167" s="3" t="n"/>
+      <c r="I167" s="3" t="n"/>
     </row>
     <row r="168">
       <c r="B168" s="2" t="n"/>
-      <c r="G168" s="3" t="n"/>
       <c r="H168" s="3" t="n"/>
+      <c r="I168" s="3" t="n"/>
     </row>
     <row r="169">
       <c r="B169" s="2" t="n"/>
-      <c r="G169" s="3" t="n"/>
       <c r="H169" s="3" t="n"/>
+      <c r="I169" s="3" t="n"/>
     </row>
     <row r="170">
       <c r="B170" s="2" t="n"/>
-      <c r="G170" s="3" t="n"/>
       <c r="H170" s="3" t="n"/>
+      <c r="I170" s="3" t="n"/>
     </row>
     <row r="171">
       <c r="B171" s="2" t="n"/>
-      <c r="G171" s="3" t="n"/>
       <c r="H171" s="3" t="n"/>
+      <c r="I171" s="3" t="n"/>
     </row>
     <row r="172">
       <c r="B172" s="2" t="n"/>
-      <c r="G172" s="3" t="n"/>
       <c r="H172" s="3" t="n"/>
+      <c r="I172" s="3" t="n"/>
     </row>
     <row r="173">
       <c r="B173" s="2" t="n"/>
-      <c r="G173" s="3" t="n"/>
       <c r="H173" s="3" t="n"/>
+      <c r="I173" s="3" t="n"/>
     </row>
     <row r="174">
       <c r="B174" s="2" t="n"/>
-      <c r="G174" s="3" t="n"/>
       <c r="H174" s="3" t="n"/>
+      <c r="I174" s="3" t="n"/>
     </row>
     <row r="175">
       <c r="B175" s="2" t="n"/>
-      <c r="G175" s="3" t="n"/>
       <c r="H175" s="3" t="n"/>
+      <c r="I175" s="3" t="n"/>
     </row>
     <row r="176">
       <c r="B176" s="2" t="n"/>
-      <c r="G176" s="3" t="n"/>
       <c r="H176" s="3" t="n"/>
+      <c r="I176" s="3" t="n"/>
     </row>
     <row r="177">
       <c r="B177" s="2" t="n"/>
-      <c r="G177" s="3" t="n"/>
       <c r="H177" s="3" t="n"/>
+      <c r="I177" s="3" t="n"/>
     </row>
     <row r="178">
       <c r="B178" s="2" t="n"/>
-      <c r="G178" s="3" t="n"/>
       <c r="H178" s="3" t="n"/>
+      <c r="I178" s="3" t="n"/>
     </row>
     <row r="179">
       <c r="B179" s="2" t="n"/>
-      <c r="G179" s="3" t="n"/>
       <c r="H179" s="3" t="n"/>
+      <c r="I179" s="3" t="n"/>
     </row>
     <row r="180">
       <c r="B180" s="2" t="n"/>
-      <c r="G180" s="3" t="n"/>
       <c r="H180" s="3" t="n"/>
+      <c r="I180" s="3" t="n"/>
     </row>
     <row r="181">
       <c r="B181" s="2" t="n"/>
-      <c r="G181" s="3" t="n"/>
       <c r="H181" s="3" t="n"/>
+      <c r="I181" s="3" t="n"/>
     </row>
     <row r="182">
       <c r="B182" s="2" t="n"/>
-      <c r="G182" s="3" t="n"/>
       <c r="H182" s="3" t="n"/>
+      <c r="I182" s="3" t="n"/>
     </row>
     <row r="183">
       <c r="B183" s="2" t="n"/>
-      <c r="G183" s="3" t="n"/>
       <c r="H183" s="3" t="n"/>
+      <c r="I183" s="3" t="n"/>
     </row>
     <row r="184">
       <c r="B184" s="2" t="n"/>
-      <c r="G184" s="3" t="n"/>
       <c r="H184" s="3" t="n"/>
+      <c r="I184" s="3" t="n"/>
     </row>
     <row r="185">
       <c r="B185" s="2" t="n"/>
-      <c r="G185" s="3" t="n"/>
       <c r="H185" s="3" t="n"/>
+      <c r="I185" s="3" t="n"/>
     </row>
     <row r="186">
       <c r="B186" s="2" t="n"/>
-      <c r="G186" s="3" t="n"/>
       <c r="H186" s="3" t="n"/>
+      <c r="I186" s="3" t="n"/>
     </row>
     <row r="187">
       <c r="B187" s="2" t="n"/>
-      <c r="G187" s="3" t="n"/>
       <c r="H187" s="3" t="n"/>
+      <c r="I187" s="3" t="n"/>
     </row>
     <row r="188">
       <c r="B188" s="2" t="n"/>
-      <c r="G188" s="3" t="n"/>
       <c r="H188" s="3" t="n"/>
+      <c r="I188" s="3" t="n"/>
     </row>
     <row r="189">
       <c r="B189" s="2" t="n"/>
-      <c r="G189" s="3" t="n"/>
       <c r="H189" s="3" t="n"/>
+      <c r="I189" s="3" t="n"/>
     </row>
     <row r="190">
       <c r="B190" s="2" t="n"/>
-      <c r="G190" s="3" t="n"/>
       <c r="H190" s="3" t="n"/>
+      <c r="I190" s="3" t="n"/>
     </row>
     <row r="191">
       <c r="B191" s="2" t="n"/>
-      <c r="G191" s="3" t="n"/>
       <c r="H191" s="3" t="n"/>
+      <c r="I191" s="3" t="n"/>
     </row>
     <row r="192">
       <c r="B192" s="2" t="n"/>
-      <c r="G192" s="3" t="n"/>
       <c r="H192" s="3" t="n"/>
+      <c r="I192" s="3" t="n"/>
     </row>
     <row r="193">
       <c r="B193" s="2" t="n"/>
-      <c r="G193" s="3" t="n"/>
       <c r="H193" s="3" t="n"/>
+      <c r="I193" s="3" t="n"/>
     </row>
     <row r="194">
       <c r="B194" s="2" t="n"/>
-      <c r="G194" s="3" t="n"/>
       <c r="H194" s="3" t="n"/>
+      <c r="I194" s="3" t="n"/>
     </row>
     <row r="195">
       <c r="B195" s="2" t="n"/>
-      <c r="G195" s="3" t="n"/>
       <c r="H195" s="3" t="n"/>
+      <c r="I195" s="3" t="n"/>
     </row>
     <row r="196">
       <c r="B196" s="2" t="n"/>
-      <c r="G196" s="3" t="n"/>
       <c r="H196" s="3" t="n"/>
+      <c r="I196" s="3" t="n"/>
     </row>
     <row r="197">
       <c r="B197" s="2" t="n"/>
-      <c r="G197" s="3" t="n"/>
       <c r="H197" s="3" t="n"/>
+      <c r="I197" s="3" t="n"/>
     </row>
     <row r="198">
       <c r="B198" s="2" t="n"/>
-      <c r="G198" s="3" t="n"/>
       <c r="H198" s="3" t="n"/>
+      <c r="I198" s="3" t="n"/>
     </row>
     <row r="199">
       <c r="B199" s="2" t="n"/>
-      <c r="G199" s="3" t="n"/>
       <c r="H199" s="3" t="n"/>
+      <c r="I199" s="3" t="n"/>
     </row>
     <row r="200">
       <c r="B200" s="2" t="n"/>
-      <c r="G200" s="3" t="n"/>
       <c r="H200" s="3" t="n"/>
+      <c r="I200" s="3" t="n"/>
     </row>
     <row r="201">
       <c r="B201" s="2" t="n"/>
-      <c r="G201" s="3" t="n"/>
       <c r="H201" s="3" t="n"/>
+      <c r="I201" s="3" t="n"/>
     </row>
     <row r="202">
       <c r="B202" s="2" t="n"/>
-      <c r="G202" s="3" t="n"/>
       <c r="H202" s="3" t="n"/>
+      <c r="I202" s="3" t="n"/>
     </row>
     <row r="203">
       <c r="B203" s="2" t="n"/>
-      <c r="G203" s="3" t="n"/>
       <c r="H203" s="3" t="n"/>
+      <c r="I203" s="3" t="n"/>
     </row>
     <row r="204">
       <c r="B204" s="2" t="n"/>
-      <c r="G204" s="3" t="n"/>
       <c r="H204" s="3" t="n"/>
+      <c r="I204" s="3" t="n"/>
     </row>
     <row r="205">
       <c r="B205" s="2" t="n"/>
-      <c r="G205" s="3" t="n"/>
       <c r="H205" s="3" t="n"/>
+      <c r="I205" s="3" t="n"/>
     </row>
     <row r="206">
       <c r="B206" s="2" t="n"/>
-      <c r="G206" s="3" t="n"/>
       <c r="H206" s="3" t="n"/>
+      <c r="I206" s="3" t="n"/>
     </row>
     <row r="207">
       <c r="B207" s="2" t="n"/>
-      <c r="G207" s="3" t="n"/>
       <c r="H207" s="3" t="n"/>
+      <c r="I207" s="3" t="n"/>
     </row>
     <row r="208">
       <c r="B208" s="2" t="n"/>
-      <c r="G208" s="3" t="n"/>
       <c r="H208" s="3" t="n"/>
+      <c r="I208" s="3" t="n"/>
     </row>
     <row r="209">
       <c r="B209" s="2" t="n"/>
-      <c r="G209" s="3" t="n"/>
       <c r="H209" s="3" t="n"/>
+      <c r="I209" s="3" t="n"/>
     </row>
     <row r="210">
       <c r="B210" s="2" t="n"/>
-      <c r="G210" s="3" t="n"/>
       <c r="H210" s="3" t="n"/>
+      <c r="I210" s="3" t="n"/>
     </row>
     <row r="211">
       <c r="B211" s="2" t="n"/>
-      <c r="G211" s="3" t="n"/>
       <c r="H211" s="3" t="n"/>
+      <c r="I211" s="3" t="n"/>
     </row>
     <row r="212">
       <c r="B212" s="2" t="n"/>
-      <c r="G212" s="3" t="n"/>
       <c r="H212" s="3" t="n"/>
+      <c r="I212" s="3" t="n"/>
     </row>
     <row r="213">
       <c r="B213" s="2" t="n"/>
-      <c r="G213" s="3" t="n"/>
       <c r="H213" s="3" t="n"/>
+      <c r="I213" s="3" t="n"/>
     </row>
     <row r="214">
       <c r="B214" s="2" t="n"/>
-      <c r="G214" s="3" t="n"/>
       <c r="H214" s="3" t="n"/>
+      <c r="I214" s="3" t="n"/>
     </row>
     <row r="215">
       <c r="B215" s="2" t="n"/>
-      <c r="G215" s="3" t="n"/>
       <c r="H215" s="3" t="n"/>
+      <c r="I215" s="3" t="n"/>
     </row>
     <row r="216">
       <c r="B216" s="2" t="n"/>
-      <c r="G216" s="3" t="n"/>
       <c r="H216" s="3" t="n"/>
+      <c r="I216" s="3" t="n"/>
     </row>
     <row r="217">
       <c r="B217" s="2" t="n"/>
-      <c r="G217" s="3" t="n"/>
       <c r="H217" s="3" t="n"/>
+      <c r="I217" s="3" t="n"/>
     </row>
     <row r="218">
       <c r="B218" s="2" t="n"/>
-      <c r="G218" s="3" t="n"/>
       <c r="H218" s="3" t="n"/>
+      <c r="I218" s="3" t="n"/>
     </row>
     <row r="219">
       <c r="B219" s="2" t="n"/>
-      <c r="G219" s="3" t="n"/>
       <c r="H219" s="3" t="n"/>
+      <c r="I219" s="3" t="n"/>
     </row>
     <row r="220">
       <c r="B220" s="2" t="n"/>
-      <c r="G220" s="3" t="n"/>
       <c r="H220" s="3" t="n"/>
+      <c r="I220" s="3" t="n"/>
     </row>
     <row r="221">
       <c r="B221" s="2" t="n"/>
-      <c r="G221" s="3" t="n"/>
       <c r="H221" s="3" t="n"/>
+      <c r="I221" s="3" t="n"/>
     </row>
     <row r="222">
       <c r="B222" s="2" t="n"/>
-      <c r="G222" s="3" t="n"/>
       <c r="H222" s="3" t="n"/>
+      <c r="I222" s="3" t="n"/>
     </row>
     <row r="223">
       <c r="B223" s="2" t="n"/>
-      <c r="G223" s="3" t="n"/>
       <c r="H223" s="3" t="n"/>
+      <c r="I223" s="3" t="n"/>
     </row>
     <row r="224">
       <c r="B224" s="2" t="n"/>
-      <c r="G224" s="3" t="n"/>
       <c r="H224" s="3" t="n"/>
+      <c r="I224" s="3" t="n"/>
     </row>
     <row r="225">
       <c r="B225" s="2" t="n"/>
-      <c r="G225" s="3" t="n"/>
       <c r="H225" s="3" t="n"/>
+      <c r="I225" s="3" t="n"/>
     </row>
     <row r="226">
       <c r="B226" s="2" t="n"/>
-      <c r="G226" s="3" t="n"/>
       <c r="H226" s="3" t="n"/>
+      <c r="I226" s="3" t="n"/>
     </row>
     <row r="227">
       <c r="B227" s="2" t="n"/>
-      <c r="G227" s="3" t="n"/>
       <c r="H227" s="3" t="n"/>
+      <c r="I227" s="3" t="n"/>
     </row>
     <row r="228">
       <c r="B228" s="2" t="n"/>
-      <c r="G228" s="3" t="n"/>
       <c r="H228" s="3" t="n"/>
+      <c r="I228" s="3" t="n"/>
     </row>
     <row r="229">
       <c r="B229" s="2" t="n"/>
-      <c r="G229" s="3" t="n"/>
       <c r="H229" s="3" t="n"/>
+      <c r="I229" s="3" t="n"/>
     </row>
     <row r="230">
       <c r="B230" s="2" t="n"/>
-      <c r="G230" s="3" t="n"/>
       <c r="H230" s="3" t="n"/>
+      <c r="I230" s="3" t="n"/>
     </row>
     <row r="231">
       <c r="B231" s="2" t="n"/>
-      <c r="G231" s="3" t="n"/>
       <c r="H231" s="3" t="n"/>
+      <c r="I231" s="3" t="n"/>
     </row>
     <row r="232">
       <c r="B232" s="2" t="n"/>
-      <c r="G232" s="3" t="n"/>
       <c r="H232" s="3" t="n"/>
+      <c r="I232" s="3" t="n"/>
     </row>
     <row r="233">
       <c r="B233" s="2" t="n"/>
-      <c r="G233" s="3" t="n"/>
       <c r="H233" s="3" t="n"/>
+      <c r="I233" s="3" t="n"/>
     </row>
     <row r="234">
       <c r="B234" s="2" t="n"/>
-      <c r="G234" s="3" t="n"/>
       <c r="H234" s="3" t="n"/>
+      <c r="I234" s="3" t="n"/>
     </row>
     <row r="235">
       <c r="B235" s="2" t="n"/>
-      <c r="G235" s="3" t="n"/>
       <c r="H235" s="3" t="n"/>
+      <c r="I235" s="3" t="n"/>
     </row>
     <row r="236">
       <c r="B236" s="2" t="n"/>
-      <c r="G236" s="3" t="n"/>
       <c r="H236" s="3" t="n"/>
+      <c r="I236" s="3" t="n"/>
     </row>
     <row r="237">
       <c r="B237" s="2" t="n"/>
-      <c r="G237" s="3" t="n"/>
       <c r="H237" s="3" t="n"/>
+      <c r="I237" s="3" t="n"/>
     </row>
     <row r="238">
       <c r="B238" s="2" t="n"/>
-      <c r="G238" s="3" t="n"/>
       <c r="H238" s="3" t="n"/>
+      <c r="I238" s="3" t="n"/>
     </row>
     <row r="239">
       <c r="B239" s="2" t="n"/>
-      <c r="G239" s="3" t="n"/>
       <c r="H239" s="3" t="n"/>
+      <c r="I239" s="3" t="n"/>
     </row>
     <row r="240">
       <c r="B240" s="2" t="n"/>
-      <c r="G240" s="3" t="n"/>
       <c r="H240" s="3" t="n"/>
+      <c r="I240" s="3" t="n"/>
     </row>
     <row r="241">
       <c r="B241" s="2" t="n"/>
-      <c r="G241" s="3" t="n"/>
       <c r="H241" s="3" t="n"/>
+      <c r="I241" s="3" t="n"/>
     </row>
     <row r="242">
       <c r="B242" s="2" t="n"/>
-      <c r="G242" s="3" t="n"/>
       <c r="H242" s="3" t="n"/>
+      <c r="I242" s="3" t="n"/>
     </row>
     <row r="243">
       <c r="B243" s="2" t="n"/>
-      <c r="G243" s="3" t="n"/>
       <c r="H243" s="3" t="n"/>
+      <c r="I243" s="3" t="n"/>
     </row>
     <row r="244">
       <c r="B244" s="2" t="n"/>
-      <c r="G244" s="3" t="n"/>
       <c r="H244" s="3" t="n"/>
+      <c r="I244" s="3" t="n"/>
     </row>
     <row r="245">
       <c r="B245" s="2" t="n"/>
-      <c r="G245" s="3" t="n"/>
       <c r="H245" s="3" t="n"/>
+      <c r="I245" s="3" t="n"/>
     </row>
     <row r="246">
       <c r="B246" s="2" t="n"/>
-      <c r="G246" s="3" t="n"/>
       <c r="H246" s="3" t="n"/>
+      <c r="I246" s="3" t="n"/>
     </row>
     <row r="247">
       <c r="B247" s="2" t="n"/>
-      <c r="G247" s="3" t="n"/>
       <c r="H247" s="3" t="n"/>
+      <c r="I247" s="3" t="n"/>
     </row>
     <row r="248">
       <c r="B248" s="2" t="n"/>
-      <c r="G248" s="3" t="n"/>
       <c r="H248" s="3" t="n"/>
+      <c r="I248" s="3" t="n"/>
     </row>
     <row r="249">
       <c r="B249" s="2" t="n"/>
-      <c r="G249" s="3" t="n"/>
       <c r="H249" s="3" t="n"/>
+      <c r="I249" s="3" t="n"/>
     </row>
     <row r="250">
       <c r="B250" s="2" t="n"/>
-      <c r="G250" s="3" t="n"/>
       <c r="H250" s="3" t="n"/>
+      <c r="I250" s="3" t="n"/>
     </row>
     <row r="251">
       <c r="B251" s="2" t="n"/>
-      <c r="G251" s="3" t="n"/>
       <c r="H251" s="3" t="n"/>
+      <c r="I251" s="3" t="n"/>
     </row>
     <row r="252">
       <c r="B252" s="2" t="n"/>
-      <c r="G252" s="3" t="n"/>
       <c r="H252" s="3" t="n"/>
+      <c r="I252" s="3" t="n"/>
     </row>
     <row r="253">
       <c r="B253" s="2" t="n"/>
-      <c r="G253" s="3" t="n"/>
       <c r="H253" s="3" t="n"/>
+      <c r="I253" s="3" t="n"/>
     </row>
     <row r="254">
       <c r="B254" s="2" t="n"/>
-      <c r="G254" s="3" t="n"/>
       <c r="H254" s="3" t="n"/>
+      <c r="I254" s="3" t="n"/>
     </row>
     <row r="255">
       <c r="B255" s="2" t="n"/>
-      <c r="G255" s="3" t="n"/>
       <c r="H255" s="3" t="n"/>
+      <c r="I255" s="3" t="n"/>
     </row>
     <row r="256">
       <c r="B256" s="2" t="n"/>
-      <c r="G256" s="3" t="n"/>
       <c r="H256" s="3" t="n"/>
+      <c r="I256" s="3" t="n"/>
     </row>
     <row r="257">
       <c r="B257" s="2" t="n"/>
-      <c r="G257" s="3" t="n"/>
       <c r="H257" s="3" t="n"/>
+      <c r="I257" s="3" t="n"/>
     </row>
     <row r="258">
       <c r="B258" s="2" t="n"/>
-      <c r="G258" s="3" t="n"/>
       <c r="H258" s="3" t="n"/>
+      <c r="I258" s="3" t="n"/>
     </row>
     <row r="259">
       <c r="B259" s="2" t="n"/>
-      <c r="G259" s="3" t="n"/>
       <c r="H259" s="3" t="n"/>
+      <c r="I259" s="3" t="n"/>
     </row>
     <row r="260">
       <c r="B260" s="2" t="n"/>
-      <c r="G260" s="3" t="n"/>
       <c r="H260" s="3" t="n"/>
+      <c r="I260" s="3" t="n"/>
     </row>
     <row r="261">
       <c r="B261" s="2" t="n"/>
-      <c r="G261" s="3" t="n"/>
       <c r="H261" s="3" t="n"/>
+      <c r="I261" s="3" t="n"/>
     </row>
     <row r="262">
       <c r="B262" s="2" t="n"/>
-      <c r="G262" s="3" t="n"/>
       <c r="H262" s="3" t="n"/>
+      <c r="I262" s="3" t="n"/>
     </row>
     <row r="263">
       <c r="B263" s="2" t="n"/>
-      <c r="G263" s="3" t="n"/>
       <c r="H263" s="3" t="n"/>
+      <c r="I263" s="3" t="n"/>
     </row>
     <row r="264">
       <c r="B264" s="2" t="n"/>
-      <c r="G264" s="3" t="n"/>
       <c r="H264" s="3" t="n"/>
+      <c r="I264" s="3" t="n"/>
     </row>
     <row r="265">
       <c r="B265" s="2" t="n"/>
-      <c r="G265" s="3" t="n"/>
       <c r="H265" s="3" t="n"/>
+      <c r="I265" s="3" t="n"/>
     </row>
     <row r="266">
       <c r="B266" s="2" t="n"/>
-      <c r="G266" s="3" t="n"/>
       <c r="H266" s="3" t="n"/>
+      <c r="I266" s="3" t="n"/>
     </row>
     <row r="267">
       <c r="B267" s="2" t="n"/>
-      <c r="G267" s="3" t="n"/>
       <c r="H267" s="3" t="n"/>
+      <c r="I267" s="3" t="n"/>
     </row>
     <row r="268">
       <c r="B268" s="2" t="n"/>
-      <c r="G268" s="3" t="n"/>
       <c r="H268" s="3" t="n"/>
+      <c r="I268" s="3" t="n"/>
     </row>
     <row r="269">
       <c r="B269" s="2" t="n"/>
-      <c r="G269" s="3" t="n"/>
       <c r="H269" s="3" t="n"/>
+      <c r="I269" s="3" t="n"/>
     </row>
     <row r="270">
       <c r="B270" s="2" t="n"/>
-      <c r="G270" s="3" t="n"/>
       <c r="H270" s="3" t="n"/>
+      <c r="I270" s="3" t="n"/>
     </row>
     <row r="271">
       <c r="B271" s="2" t="n"/>
-      <c r="G271" s="3" t="n"/>
       <c r="H271" s="3" t="n"/>
+      <c r="I271" s="3" t="n"/>
     </row>
     <row r="272">
       <c r="B272" s="2" t="n"/>
-      <c r="G272" s="3" t="n"/>
       <c r="H272" s="3" t="n"/>
+      <c r="I272" s="3" t="n"/>
     </row>
     <row r="273">
       <c r="B273" s="2" t="n"/>
-      <c r="G273" s="3" t="n"/>
       <c r="H273" s="3" t="n"/>
+      <c r="I273" s="3" t="n"/>
     </row>
     <row r="274">
       <c r="B274" s="2" t="n"/>
-      <c r="G274" s="3" t="n"/>
       <c r="H274" s="3" t="n"/>
+      <c r="I274" s="3" t="n"/>
     </row>
     <row r="275">
       <c r="B275" s="2" t="n"/>
-      <c r="G275" s="3" t="n"/>
       <c r="H275" s="3" t="n"/>
+      <c r="I275" s="3" t="n"/>
     </row>
     <row r="276">
       <c r="B276" s="2" t="n"/>
-      <c r="G276" s="3" t="n"/>
       <c r="H276" s="3" t="n"/>
+      <c r="I276" s="3" t="n"/>
     </row>
     <row r="277">
       <c r="B277" s="2" t="n"/>
-      <c r="G277" s="3" t="n"/>
       <c r="H277" s="3" t="n"/>
+      <c r="I277" s="3" t="n"/>
     </row>
     <row r="278">
       <c r="B278" s="2" t="n"/>
-      <c r="G278" s="3" t="n"/>
       <c r="H278" s="3" t="n"/>
+      <c r="I278" s="3" t="n"/>
     </row>
     <row r="279">
       <c r="B279" s="2" t="n"/>
-      <c r="G279" s="3" t="n"/>
       <c r="H279" s="3" t="n"/>
+      <c r="I279" s="3" t="n"/>
     </row>
     <row r="280">
       <c r="B280" s="2" t="n"/>
-      <c r="G280" s="3" t="n"/>
       <c r="H280" s="3" t="n"/>
+      <c r="I280" s="3" t="n"/>
     </row>
     <row r="281">
       <c r="B281" s="2" t="n"/>
-      <c r="G281" s="3" t="n"/>
       <c r="H281" s="3" t="n"/>
+      <c r="I281" s="3" t="n"/>
     </row>
     <row r="282">
       <c r="B282" s="2" t="n"/>
-      <c r="G282" s="3" t="n"/>
       <c r="H282" s="3" t="n"/>
+      <c r="I282" s="3" t="n"/>
     </row>
     <row r="283">
       <c r="B283" s="2" t="n"/>
-      <c r="G283" s="3" t="n"/>
       <c r="H283" s="3" t="n"/>
+      <c r="I283" s="3" t="n"/>
     </row>
     <row r="284">
       <c r="B284" s="2" t="n"/>
-      <c r="G284" s="3" t="n"/>
       <c r="H284" s="3" t="n"/>
+      <c r="I284" s="3" t="n"/>
     </row>
     <row r="285">
       <c r="B285" s="2" t="n"/>
-      <c r="G285" s="3" t="n"/>
       <c r="H285" s="3" t="n"/>
+      <c r="I285" s="3" t="n"/>
     </row>
     <row r="286">
       <c r="B286" s="2" t="n"/>
-      <c r="G286" s="3" t="n"/>
       <c r="H286" s="3" t="n"/>
+      <c r="I286" s="3" t="n"/>
     </row>
     <row r="287">
       <c r="B287" s="2" t="n"/>
-      <c r="G287" s="3" t="n"/>
       <c r="H287" s="3" t="n"/>
+      <c r="I287" s="3" t="n"/>
     </row>
     <row r="288">
       <c r="B288" s="2" t="n"/>
-      <c r="G288" s="3" t="n"/>
       <c r="H288" s="3" t="n"/>
+      <c r="I288" s="3" t="n"/>
     </row>
     <row r="289">
       <c r="B289" s="2" t="n"/>
-      <c r="G289" s="3" t="n"/>
       <c r="H289" s="3" t="n"/>
+      <c r="I289" s="3" t="n"/>
     </row>
     <row r="290">
       <c r="B290" s="2" t="n"/>
-      <c r="G290" s="3" t="n"/>
       <c r="H290" s="3" t="n"/>
+      <c r="I290" s="3" t="n"/>
     </row>
     <row r="291">
       <c r="B291" s="2" t="n"/>
-      <c r="G291" s="3" t="n"/>
       <c r="H291" s="3" t="n"/>
+      <c r="I291" s="3" t="n"/>
     </row>
     <row r="292">
       <c r="B292" s="2" t="n"/>
-      <c r="G292" s="3" t="n"/>
       <c r="H292" s="3" t="n"/>
+      <c r="I292" s="3" t="n"/>
     </row>
     <row r="293">
       <c r="B293" s="2" t="n"/>
-      <c r="G293" s="3" t="n"/>
       <c r="H293" s="3" t="n"/>
+      <c r="I293" s="3" t="n"/>
     </row>
     <row r="294">
       <c r="B294" s="2" t="n"/>
-      <c r="G294" s="3" t="n"/>
       <c r="H294" s="3" t="n"/>
+      <c r="I294" s="3" t="n"/>
     </row>
     <row r="295">
       <c r="B295" s="2" t="n"/>
-      <c r="G295" s="3" t="n"/>
       <c r="H295" s="3" t="n"/>
+      <c r="I295" s="3" t="n"/>
     </row>
     <row r="296">
       <c r="B296" s="2" t="n"/>
-      <c r="G296" s="3" t="n"/>
       <c r="H296" s="3" t="n"/>
+      <c r="I296" s="3" t="n"/>
     </row>
     <row r="297">
       <c r="B297" s="2" t="n"/>
-      <c r="G297" s="3" t="n"/>
       <c r="H297" s="3" t="n"/>
+      <c r="I297" s="3" t="n"/>
     </row>
     <row r="298">
       <c r="B298" s="2" t="n"/>
-      <c r="G298" s="3" t="n"/>
       <c r="H298" s="3" t="n"/>
+      <c r="I298" s="3" t="n"/>
     </row>
     <row r="299">
       <c r="B299" s="2" t="n"/>
-      <c r="G299" s="3" t="n"/>
       <c r="H299" s="3" t="n"/>
+      <c r="I299" s="3" t="n"/>
     </row>
     <row r="300">
       <c r="B300" s="2" t="n"/>
-      <c r="G300" s="3" t="n"/>
       <c r="H300" s="3" t="n"/>
+      <c r="I300" s="3" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"景点,早餐,午餐,晚餐,住宿,交通,其他,标题"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2284,16 +2411,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>第一个工作表“行程”：每一行是一个地点。</t>
+          <t>第一个工作表“行程”：每一行是一个地点、一餐、一个住宿或一段交通。</t>
         </is>
       </c>
     </row>
@@ -2307,40 +2434,54 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>时间：例如 09:30，可以留空。同一天里按时间排序。</t>
+          <t>时间：例如 09:30，可以留空。同一天里按时间排序；早餐、午餐、晚餐、住宿留空时会排在合适的位置。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>地点：必填。没有地点名称的行会被忽略。</t>
+          <t>类别：景点、早餐、午餐、晚餐、住宿、交通、其他、标题。留空按景点处理。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>城市、地址、备注：随便填。城市写中文（例如 西安），地图会用它估算位置。</t>
+          <t>标题：这一行的“地点”会作为当天的标题，“备注”作为标题下的说明。不填标题时，标题由当天景点的名字自动连起来。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>纬度、经度：可以留空。在 Google 地图上右键点地点，就能复制。</t>
+          <t>地点：必填。没有地点名称的行会被忽略。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>第二个工作表“设置”：行程名称和出发日期。</t>
+          <t>城市、地址、备注：随便填。城市写中文（例如 西安），地图会用它估算位置。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>纬度、经度：可以留空。在 Google 地图上右键点地点，就能复制。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>第二个工作表“设置”：行程名称和出发日期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>示例行程（备注以“示例”开头）请删掉，换成你们自己的。</t>
         </is>

</xml_diff>